<commit_message>
Add America, Europe, Australia regions and upgrade to 20 workers
</commit_message>
<xml_diff>
--- a/output/leads_latest.xlsx
+++ b/output/leads_latest.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG3"/>
+  <dimension ref="A1:AG19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -636,12 +636,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FOOTDISTRICT</t>
+          <t>Dictionary</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://footdistrict.com</t>
+          <t>https://dictionary.cambridge.org</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -649,80 +649,2480 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>help@footdistrict.com</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Verified (Deliverable)</t>
+          <t>Unverified</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='dictionary.cambridge.org</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Idea for Dictionary (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Hi Dictionary Team,
+Love what you've built with Dictionary—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org, leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Dictionary?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Quick observation on Dictionary's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Hi Dictionary Team,
+Quick note regarding Dictionary—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Dictionary (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Hi Dictionary Team,
+I put together a quick technical audit for Dictionary. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>2-min video for Dictionary?</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Hi Dictionary Team,
+Spotted a quick fix on Dictionary's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Dictionary. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Dictionary—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Dictionary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>2026-08-16 21:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mybest</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://vn.my-best.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>1533</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1533ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Idea for mybest (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Hi mybest Team,
+Love what you've built with mybest—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for mybest?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Quick observation on mybest's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Hi mybest Team,
+Quick note regarding mybest—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for mybest (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Hi mybest Team,
+I put together a quick technical audit for mybest. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>2-min video for mybest?</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Hi mybest Team,
+Spotted a quick fix on mybest's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at mybest. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for mybest—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at mybest. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Merriam-webster</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://merriam-webster.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>3523</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3523ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Idea for Merriam-webster (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Hi Merriam-webster Team,
+Love what you've built with Merriam-webster—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Merriam-webster?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Quick observation on Merriam-webster's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Hi Merriam-webster Team,
+Quick note regarding Merriam-webster—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Merriam-webster (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Hi Merriam-webster Team,
+I put together a quick technical audit for Merriam-webster. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>2-min video for Merriam-webster?</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Hi Merriam-webster Team,
+Spotted a quick fix on Merriam-webster's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Merriam-webster. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Merriam-webster—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Merriam-webster. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BEST Express Vietnam</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://sale.best-inc.vn</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>19001031</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>@bestexpressvietnam</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bestexpressvietnam/</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/bestexpressvietnam/</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>1724</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1724ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express Vietnam?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>2-min video for BEST Express Vietnam?</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BEST Express Vietnam</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://service.best-inc.vn</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mkt-vn-sns@best-inc.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>19001031</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>@bestexpressvietnam</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bestexpressvietnam/</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/bestexpressvietnam</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>1829</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1829ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express Vietnam?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>2-min video for BEST Express Vietnam?</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Vietnam Team,
+Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>Contacted</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BEST Express</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://best-inc.vn</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fullpage.js@2.9.7</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Undeliverable Domain</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Custom / Headless</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>4226</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4226ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Idea for BEST Express (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Team,
+Love what you've built with BEST Express—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Quick observation on BEST Express's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Team,
+Quick note regarding BEST Express—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for BEST Express (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Team,
+I put together a quick technical audit for BEST Express. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>2-min video for BEST Express?</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Hi BEST Express Team,
+Spotted a quick fix on BEST Express's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at BEST Express. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at BEST Express. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Synonyms and Antonyms of Words</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://thesaurus.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>@dictionarycom</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dictionarycom</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dictionarycom</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>WooCommerce / WordPress</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>4121</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4121ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Idea for Synonyms and Antonyms of Words (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Hi Synonyms and Antonyms of Words Team,
+Love what you've built with Synonyms and Antonyms of Words—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Synonyms and Antonyms of Words?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Quick observation on Synonyms and Antonyms of Words's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Hi Synonyms and Antonyms of Words Team,
+Quick note regarding Synonyms and Antonyms of Words—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Synonyms and Antonyms of Words (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Hi Synonyms and Antonyms of Words Team,
+I put together a quick technical audit for Synonyms and Antonyms of Words. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>2-min video for Synonyms and Antonyms of Words?</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>Hi Synonyms and Antonyms of Words Team,
+Spotted a quick fix on Synonyms and Antonyms of Words's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Synonyms and Antonyms of Words. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Synonyms and Antonyms of Words—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Synonyms and Antonyms of Words. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Umbrex</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://umbrex.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Custom / Headless</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>4225</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4225ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Idea for Umbrex (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+Love what you've built with Umbrex—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Umbrex?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Quick observation on Umbrex's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+Quick note regarding Umbrex—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Umbrex (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+I put together a quick technical audit for Umbrex. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>2-min video for Umbrex?</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+Spotted a quick fix on Umbrex's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Umbrex. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Umbrex—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Umbrex. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Onlinelibrary</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>970</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Idea for Onlinelibrary (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Love what you've built with Onlinelibrary—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Onlinelibrary?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Quick observation on Onlinelibrary's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Quick note regarding Onlinelibrary—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Onlinelibrary (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+I put together a quick technical audit for Onlinelibrary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>2-min video for Onlinelibrary?</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Spotted a quick fix on Onlinelibrary's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Onlinelibrary. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Onlinelibrary—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Onlinelibrary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Famousfootwear</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://famousfootwear.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>1238</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Idea for Famousfootwear (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+Love what you've built with Famousfootwear—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Famousfootwear?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>Quick observation on Famousfootwear's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+Quick note regarding Famousfootwear—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Famousfootwear (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+I put together a quick technical audit for Famousfootwear. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>2-min video for Famousfootwear?</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+Spotted a quick fix on Famousfootwear's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Famousfootwear. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Famousfootwear—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Famousfootwear. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Footwear etc.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://footwearetc.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>privacy@footwearetc.com</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1-800-720-0572</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>@footwearetc</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/footwearetc/</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>http://www.facebook.com/footwearetc</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>2726</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | Slow server response time (2726ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Idea for Footwear etc. (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+Love what you've built with Footwear etc.—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Footwear etc.?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Quick observation on Footwear etc.'s conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+Quick note regarding Footwear etc.—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Footwear etc. (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+I put together a quick technical audit for Footwear etc.. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>2-min video for Footwear etc.?</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+Spotted a quick fix on Footwear etc.'s checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Footwear etc.. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Footwear etc.—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Footwear etc.. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>StartUs Insights</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://startus-insights.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>zlibjs@0.3.1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Undeliverable Domain</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>WooCommerce / WordPress</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>1546</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1546ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Idea for StartUs Insights (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+Love what you've built with StartUs Insights—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for StartUs Insights?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>Quick observation on StartUs Insights's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+Quick note regarding StartUs Insights—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for StartUs Insights (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+I put together a quick technical audit for StartUs Insights. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>2-min video for StartUs Insights?</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+Spotted a quick fix on StartUs Insights's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at StartUs Insights. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for StartUs Insights—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at StartUs Insights. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Brand House Direct</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://brandhousedirect.com.au</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>support@brandhousedirect.com.au</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1300735786</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>@brandhousedirectau</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/brandhousedirectau/</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/brandhousedirect</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Custom / Headless</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>2323</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2323ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Idea for Brand House Direct (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+Love what you've built with Brand House Direct—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Brand House Direct?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>Quick observation on Brand House Direct's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+Quick note regarding Brand House Direct—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Brand House Direct (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+I put together a quick technical audit for Brand House Direct. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>2-min video for Brand House Direct?</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+Spotted a quick fix on Brand House Direct's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Brand House Direct. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brand House Direct—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Brand House Direct. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bestbuy</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://bestbuy.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.bestbuy.com', port=4</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Idea for Bestbuy (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Love what you've built with Bestbuy—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Bestbuy?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Quick observation on Bestbuy's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Quick note regarding Bestbuy—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Bestbuy (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+I put together a quick technical audit for Bestbuy. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>2-min video for Bestbuy?</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Spotted a quick fix on Bestbuy's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Bestbuy. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Bestbuy—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Bestbuy. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Myntra</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://myntra.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.myntra.com', port=44</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Idea for Myntra (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+Love what you've built with Myntra—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Myntra?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>Quick observation on Myntra's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+Quick note regarding Myntra—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Myntra (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+I put together a quick technical audit for Myntra. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>2-min video for Myntra?</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+Spotted a quick fix on Myntra's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Myntra. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Myntra—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Myntra. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Brandname.com</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://brandname.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>2220</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2220ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Idea for Brandname.com (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Hi Brandname.com Team,
+Love what you've built with Brandname.com—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Brandname.com?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Quick observation on Brandname.com's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Hi Brandname.com Team,
+Quick note regarding Brandname.com—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Brandname.com (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Hi Brandname.com Team,
+I put together a quick technical audit for Brandname.com. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>2-min video for Brandname.com?</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Hi Brandname.com Team,
+Spotted a quick fix on Brandname.com's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Brandname.com. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brandname.com—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Brandname.com. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>FOOTDISTRICT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://footdistrict.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>help@footdistrict.com</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
         <is>
           <t>@footdistrict</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>https://www.instagram.com/footdistrict/</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>https://www.facebook.com/footDistrict</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>@footdistrict</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="O2" t="n">
+      <c r="O18" t="n">
         <v>1434</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S18" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>Trustpilot</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
         <is>
           <t>Idea for FOOTDISTRICT (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 Love what you've built with FOOTDISTRICT—your site design and positioning look great. While auditing the store, I noticed product page social proof and mobile retargeting, leaving easy revenue on the table.
@@ -732,12 +3132,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>Quick observation on FOOTDISTRICT's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Y18" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 Quick note regarding FOOTDISTRICT—spotted a quick tracking and conversion gap: product page social proof and mobile retargeting, which might be causing paid traffic to bounce without converting.
@@ -747,12 +3147,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z18" t="inlineStr">
         <is>
           <t>Quick CRO fix for FOOTDISTRICT (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA18" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 I put together a quick technical audit for FOOTDISTRICT. Your page speed and branding look solid, but you're leaving revenue on the table due to product page social proof and mobile retargeting.
@@ -762,12 +3162,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB18" t="inlineStr">
         <is>
           <t>2-min video for FOOTDISTRICT?</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AC18" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 Spotted a quick fix on FOOTDISTRICT's checkout &amp; tracking setup (product page social proof and mobile retargeting). 
@@ -776,113 +3176,113 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AD18" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at FOOTDISTRICT. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for FOOTDISTRICT—would love to connect!</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AE18" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at FOOTDISTRICT. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Contacted</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
         <is>
           <t>2026-08-16 20:51</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>APB</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>https://www.apbstore.com</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>info@apbstore.com</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Verified (Deliverable)</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
         <is>
           <t>@apbstore</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>https://www.instagram.com/apbstore/?hl=en</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://www.facebook.com/theapbstore/</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="O3" t="n">
+      <c r="O19" t="n">
         <v>1021</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
         <is>
           <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>Idea for APB (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>Hi APB Team,
 Love what you've built with APB—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
@@ -892,12 +3292,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>Quick observation on APB's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y19" t="inlineStr">
         <is>
           <t>Hi APB Team,
 Quick note regarding APB—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
@@ -907,12 +3307,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z19" t="inlineStr">
         <is>
           <t>Quick CRO fix for APB (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA19" t="inlineStr">
         <is>
           <t>Hi APB Team,
 I put together a quick technical audit for APB. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
@@ -922,12 +3322,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AB19" t="inlineStr">
         <is>
           <t>2-min video for APB?</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AC19" t="inlineStr">
         <is>
           <t>Hi APB Team,
 Spotted a quick fix on APB's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
@@ -936,22 +3336,22 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AD19" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at APB. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for APB—would love to connect!</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AE19" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at APB. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AF19" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AG19" t="inlineStr">
         <is>
           <t>2026-08-16 20:48</t>
         </is>

</xml_diff>

<commit_message>
Fix lead loader on Vercel: bundle default output and sync batch response
</commit_message>
<xml_diff>
--- a/output/leads_latest.xlsx
+++ b/output/leads_latest.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG19"/>
+  <dimension ref="A1:AG24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -636,12 +636,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dictionary</t>
+          <t>Topcv</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://dictionary.cambridge.org</t>
+          <t>https://topcv.vn</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -652,7 +652,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Unverified</t>
+          <t>No Email</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -665,11 +665,11 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>688</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -694,33 +694,33 @@
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Could not connect or site timed out: HTTPSConnectionPool(host='dictionary.cambridge.org</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Idea for Dictionary (scaled UK brand from £4.6k to £696k+)</t>
+          <t>Idea for Topcv (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Hi Dictionary Team,
-Love what you've built with Dictionary—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org, leaving easy revenue on the table.
+          <t>Hi Topcv Team,
+Love what you've built with Topcv—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Dictionary?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Topcv?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Quick observation on Dictionary's conversion &amp; tracking</t>
+          <t>Quick observation on Topcv's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Hi Dictionary Team,
-Quick note regarding Dictionary—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org, which might be causing paid traffic to bounce without converting.
+          <t>Hi Topcv Team,
+Quick note regarding Topcv—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -729,13 +729,13 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Dictionary (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Topcv (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Hi Dictionary Team,
-I put together a quick technical audit for Dictionary. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org.
+          <t>Hi Topcv Team,
+I put together a quick technical audit for Topcv. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -744,13 +744,13 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2-min video for Dictionary?</t>
+          <t>2-min video for Topcv?</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>Hi Dictionary Team,
-Spotted a quick fix on Dictionary's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='dictionary.cambridge.org). 
+          <t>Hi Topcv Team,
+Spotted a quick fix on Topcv's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -758,12 +758,12 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Dictionary. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Dictionary—would love to connect!</t>
+          <t>Hi there, love what you're building at Topcv. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Topcv—would love to connect!</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Dictionary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Topcv. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -773,24 +773,24 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>2026-08-16 21:05</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mybest</t>
+          <t>Cambridge Dictionary</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://vn.my-best.com</t>
+          <t>https://dictionary.cambridge.org</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -803,9 +803,21 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>@cambridgewords</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/cambridgewords</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/CUPCambridgeDictionary/</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
@@ -813,11 +825,11 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>1533</v>
+        <v>917</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -838,33 +850,33 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1533ms) hurting mobile conversion rate</t>
+          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Idea for mybest (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Cambridge Dictionary (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Hi mybest Team,
-Love what you've built with mybest—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for mybest?
+          <t>Hi Cambridge Dictionary Team,
+Love what you've built with Cambridge Dictionary—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Cambridge Dictionary?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Quick observation on mybest's conversion &amp; tracking</t>
+          <t>Quick observation on Cambridge Dictionary's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Hi mybest Team,
-Quick note regarding mybest—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Cambridge Dictionary Team,
+Quick note regarding Cambridge Dictionary—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -873,13 +885,13 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Quick CRO fix for mybest (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Cambridge Dictionary (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Hi mybest Team,
-I put together a quick technical audit for mybest. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Cambridge Dictionary Team,
+I put together a quick technical audit for Cambridge Dictionary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -888,13 +900,13 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>2-min video for mybest?</t>
+          <t>2-min video for Cambridge Dictionary?</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>Hi mybest Team,
-Spotted a quick fix on mybest's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Cambridge Dictionary Team,
+Spotted a quick fix on Cambridge Dictionary's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -902,12 +914,12 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at mybest. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for mybest—would love to connect!</t>
+          <t>Hi there, love what you're building at Cambridge Dictionary. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Cambridge Dictionary—would love to connect!</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at mybest. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Cambridge Dictionary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -917,51 +929,71 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Merriam-webster</t>
+          <t>Footwear etc.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://merriam-webster.com</t>
+          <t>https://footwearetc.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>privacy@footwearetc.com</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>No Email</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1-800-720-0572</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>@footwearetc</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/footwearetc/</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>http://www.facebook.com/footwearetc</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Shopify</t>
         </is>
       </c>
       <c r="O4" t="n">
-        <v>3523</v>
+        <v>3451</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -971,41 +1003,185 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3523ms) hurting mobile conversion rate</t>
+          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | Slow server response time (3451ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Idea for Merriam-webster (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Footwear etc. (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+Love what you've built with Footwear etc.—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Footwear etc.?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Quick observation on Footwear etc.'s conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+Quick note regarding Footwear etc.—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Footwear etc. (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+I put together a quick technical audit for Footwear etc.. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>2-min video for Footwear etc.?</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Hi Footwear etc. Team,
+Spotted a quick fix on Footwear etc.'s checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Footwear etc.. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Footwear etc.—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Footwear etc.. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>2026-08-16 21:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Merriam-webster</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://merriam-webster.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>3002</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3002ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Idea for Merriam-webster (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
         <is>
           <t>Hi Merriam-webster Team,
 Love what you've built with Merriam-webster—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
 Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Merriam-webster?
 Best,
 Talha</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>Quick observation on Merriam-webster's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Hi Merriam-webster Team,
 Quick note regarding Merriam-webster—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -1015,12 +1191,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>Quick CRO fix for Merriam-webster (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>Hi Merriam-webster Team,
 I put together a quick technical audit for Merriam-webster. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -1030,12 +1206,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>2-min video for Merriam-webster?</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>Hi Merriam-webster Team,
 Spotted a quick fix on Merriam-webster's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -1044,236 +1220,56 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at Merriam-webster. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Merriam-webster—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Merriam-webster. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Merriam-webster—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Merriam-webster. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>2026-08-16 20:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BEST Express Vietnam</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://sale.best-inc.vn</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>No Email</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>19001031</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>@bestexpressvietnam</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/bestexpressvietnam/</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/bestexpressvietnam/</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Magento</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>1724</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>ACTIVE ✅</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1724ms) hurting mobile conversion rate</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Hi BEST Express Vietnam Team,
-Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express Vietnam?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>Hi BEST Express Vietnam Team,
-Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>Hi BEST Express Vietnam Team,
-I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>2-min video for BEST Express Vietnam?</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Hi BEST Express Vietnam Team,
-Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BEST Express Vietnam</t>
+          <t>Famousfootwear</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://service.best-inc.vn</t>
+          <t>https://famousfootwear.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>mkt-vn-sns@best-inc.com</t>
-        </is>
-      </c>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Verified (Deliverable)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>19001031</t>
-        </is>
-      </c>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>@bestexpressvietnam</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/bestexpressvietnam/</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/bestexpressvietnam</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
@@ -1281,7 +1277,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>1829</v>
+        <v>3322</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1295,7 +1291,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1306,33 +1302,33 @@
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1829ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3322ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Famousfootwear (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Hi BEST Express Vietnam Team,
-Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express Vietnam?
+          <t>Hi Famousfootwear Team,
+Love what you've built with Famousfootwear—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Famousfootwear?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
+          <t>Quick observation on Famousfootwear's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Hi BEST Express Vietnam Team,
-Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Famousfootwear Team,
+Quick note regarding Famousfootwear—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1341,13 +1337,13 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Famousfootwear (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Hi BEST Express Vietnam Team,
-I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Famousfootwear Team,
+I put together a quick technical audit for Famousfootwear. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1356,13 +1352,13 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2-min video for BEST Express Vietnam?</t>
+          <t>2-min video for Famousfootwear?</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>Hi BEST Express Vietnam Team,
-Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Famousfootwear Team,
+Spotted a quick fix on Famousfootwear's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1370,49 +1366,49 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
+          <t>Hi there, love what you're building at Famousfootwear. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Famousfootwear—would love to connect!</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Famousfootwear. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>Contacted</t>
+          <t>New Lead</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BEST Express</t>
+          <t>Top Hotel - Official Site</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://best-inc.vn</t>
+          <t>https://tophotel.com.vn</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>fullpage.js@2.9.7</t>
+          <t>tophotel.sales@gmail.com</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Undeliverable Domain</t>
+          <t>Verified (Deliverable)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1421,19 +1417,23 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100035513540432</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Custom / Headless</t>
+          <t>WooCommerce / WordPress</t>
         </is>
       </c>
       <c r="O7" t="n">
-        <v>4226</v>
+        <v>4259</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1454,33 +1454,33 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4226ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4259ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Idea for BEST Express (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Top Hotel - Official Site (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Hi BEST Express Team,
-Love what you've built with BEST Express—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express?
+          <t>Hi Top Hotel - Official Site Team,
+Love what you've built with Top Hotel - Official Site—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Top Hotel - Official Site?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Quick observation on BEST Express's conversion &amp; tracking</t>
+          <t>Quick observation on Top Hotel - Official Site's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Hi BEST Express Team,
-Quick note regarding BEST Express—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
+          <t>Hi Top Hotel - Official Site Team,
+Quick note regarding Top Hotel - Official Site—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1489,13 +1489,13 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>Quick CRO fix for BEST Express (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Top Hotel - Official Site (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Hi BEST Express Team,
-I put together a quick technical audit for BEST Express. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
+          <t>Hi Top Hotel - Official Site Team,
+I put together a quick technical audit for Top Hotel - Official Site. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1504,13 +1504,13 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>2-min video for BEST Express?</t>
+          <t>2-min video for Top Hotel - Official Site?</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>Hi BEST Express Team,
-Spotted a quick fix on BEST Express's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
+          <t>Hi Top Hotel - Official Site Team,
+Spotted a quick fix on Top Hotel - Official Site's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1518,12 +1518,12 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at BEST Express. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express—would love to connect!</t>
+          <t>Hi there, love what you're building at Top Hotel - Official Site. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Top Hotel - Official Site—would love to connect!</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at BEST Express. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Top Hotel - Official Site. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -1533,30 +1533,34 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Synonyms and Antonyms of Words</t>
+          <t>Esquire</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://thesaurus.com</t>
+          <t>https://esquire.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>editor@esquire.com</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>No Email</t>
+          <t>Verified (Deliverable)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1565,27 +1569,31 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>@dictionarycom</t>
+          <t>@esquire</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/dictionarycom</t>
+          <t>http://instagram.com/esquire</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dictionarycom</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
+          <t>https://www.facebook.com/Esquire</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>@esquire</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>WooCommerce / WordPress</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O8" t="n">
-        <v>4121</v>
+        <v>1086</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1599,7 +1607,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1610,33 +1618,33 @@
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4121ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Idea for Synonyms and Antonyms of Words (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Esquire (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>Hi Synonyms and Antonyms of Words Team,
-Love what you've built with Synonyms and Antonyms of Words—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Synonyms and Antonyms of Words?
+          <t>Hi Esquire Team,
+Love what you've built with Esquire—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Esquire?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Quick observation on Synonyms and Antonyms of Words's conversion &amp; tracking</t>
+          <t>Quick observation on Esquire's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Hi Synonyms and Antonyms of Words Team,
-Quick note regarding Synonyms and Antonyms of Words—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Esquire Team,
+Quick note regarding Esquire—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1645,13 +1653,13 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Synonyms and Antonyms of Words (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Esquire (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Hi Synonyms and Antonyms of Words Team,
-I put together a quick technical audit for Synonyms and Antonyms of Words. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Esquire Team,
+I put together a quick technical audit for Esquire. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1660,13 +1668,13 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>2-min video for Synonyms and Antonyms of Words?</t>
+          <t>2-min video for Esquire?</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>Hi Synonyms and Antonyms of Words Team,
-Spotted a quick fix on Synonyms and Antonyms of Words's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Esquire Team,
+Spotted a quick fix on Esquire's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1674,12 +1682,12 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Synonyms and Antonyms of Words. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Synonyms and Antonyms of Words—would love to connect!</t>
+          <t>Hi there, love what you're building at Esquire. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Esquire—would love to connect!</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Synonyms and Antonyms of Words. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Esquire. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1689,47 +1697,67 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Umbrex</t>
+          <t>ELLE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://umbrex.com</t>
+          <t>https://elle.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>contactus@elle.com</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>No Email</t>
+          <t>Verified (Deliverable)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>@elleusa</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>http://instagram.com/elleusa</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ellemagazine</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>@ellemagazine</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Custom / Headless</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O9" t="n">
-        <v>4225</v>
+        <v>820</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1754,33 +1782,33 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4225ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Idea for Umbrex (scaled US store to 4.89% CVR)</t>
+          <t>Idea for ELLE (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Hi Umbrex Team,
-Love what you've built with Umbrex—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Umbrex?
+          <t>Hi ELLE Team,
+Love what you've built with ELLE—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for ELLE?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Quick observation on Umbrex's conversion &amp; tracking</t>
+          <t>Quick observation on ELLE's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Hi Umbrex Team,
-Quick note regarding Umbrex—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi ELLE Team,
+Quick note regarding ELLE—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1789,13 +1817,13 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Umbrex (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for ELLE (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Hi Umbrex Team,
-I put together a quick technical audit for Umbrex. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi ELLE Team,
+I put together a quick technical audit for ELLE. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1804,13 +1832,13 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2-min video for Umbrex?</t>
+          <t>2-min video for ELLE?</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>Hi Umbrex Team,
-Spotted a quick fix on Umbrex's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi ELLE Team,
+Spotted a quick fix on ELLE's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1818,12 +1846,12 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Umbrex. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Umbrex—would love to connect!</t>
+          <t>Hi there, love what you're building at ELLE. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for ELLE—would love to connect!</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Umbrex. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at ELLE. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -1833,24 +1861,24 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Onlinelibrary</t>
+          <t>Tops Market</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com</t>
+          <t>https://topsmarket.vn</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -1863,17 +1891,29 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>@topsmarketvn</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/topsmarketvn/</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/TopsmarketVietnam</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>WooCommerce / WordPress</t>
         </is>
       </c>
       <c r="O10" t="n">
-        <v>970</v>
+        <v>1297</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1887,7 +1927,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1898,33 +1938,33 @@
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Idea for Onlinelibrary (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Tops Market (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-Love what you've built with Onlinelibrary—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Onlinelibrary?
+          <t>Hi Tops Market Team,
+Love what you've built with Tops Market—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Tops Market?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Quick observation on Onlinelibrary's conversion &amp; tracking</t>
+          <t>Quick observation on Tops Market's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-Quick note regarding Onlinelibrary—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Tops Market Team,
+Quick note regarding Tops Market—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1933,13 +1973,13 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Onlinelibrary (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Tops Market (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-I put together a quick technical audit for Onlinelibrary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Tops Market Team,
+I put together a quick technical audit for Tops Market. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1948,13 +1988,13 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>2-min video for Onlinelibrary?</t>
+          <t>2-min video for Tops Market?</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-Spotted a quick fix on Onlinelibrary's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Tops Market Team,
+Spotted a quick fix on Tops Market's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1962,12 +2002,12 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Onlinelibrary. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Onlinelibrary—would love to connect!</t>
+          <t>Hi there, love what you're building at Tops Market. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Tops Market—would love to connect!</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Onlinelibrary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Tops Market. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -1977,24 +2017,24 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Famousfootwear</t>
+          <t>Myntra</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://famousfootwear.com</t>
+          <t>https://myntra.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -2013,11 +2053,11 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O11" t="n">
-        <v>1238</v>
+        <v>0</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -2042,33 +2082,33 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.myntra.com', port=44</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Idea for Famousfootwear (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Myntra (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-Love what you've built with Famousfootwear—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Famousfootwear?
+          <t>Hi Myntra Team,
+Love what you've built with Myntra—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Myntra?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Quick observation on Famousfootwear's conversion &amp; tracking</t>
+          <t>Quick observation on Myntra's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-Quick note regarding Famousfootwear—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Myntra Team,
+Quick note regarding Myntra—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -2077,13 +2117,13 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Famousfootwear (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Myntra (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-I put together a quick technical audit for Famousfootwear. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Myntra Team,
+I put together a quick technical audit for Myntra. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44.
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -2092,13 +2132,13 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>2-min video for Famousfootwear?</t>
+          <t>2-min video for Myntra?</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-Spotted a quick fix on Famousfootwear's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Myntra Team,
+Spotted a quick fix on Myntra's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -2106,12 +2146,12 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Famousfootwear. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Famousfootwear—would love to connect!</t>
+          <t>Hi there, love what you're building at Myntra. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Myntra—would love to connect!</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Famousfootwear. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Myntra. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -2121,19 +2161,19 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>2026-08-16 20:59</t>
+          <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Footwear etc.</t>
+          <t>mybest</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://footwearetc.com</t>
+          <t>https://vn.my-best.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2141,98 +2181,78 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>privacy@footwearetc.com</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Verified (Deliverable)</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1-800-720-0572</t>
-        </is>
-      </c>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>@footwearetc</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/footwearetc/</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>http://www.facebook.com/footwearetc</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Shopify</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O12" t="n">
-        <v>2726</v>
+        <v>1533</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>ACTIVE ✅</t>
-        </is>
-      </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | Slow server response time (2726ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1533ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Idea for Footwear etc. (scaled US store to 4.89% CVR)</t>
+          <t>Idea for mybest (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Hi Footwear etc. Team,
-Love what you've built with Footwear etc.—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
+          <t>Hi mybest Team,
+Love what you've built with mybest—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Footwear etc.?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for mybest?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Quick observation on Footwear etc.'s conversion &amp; tracking</t>
+          <t>Quick observation on mybest's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Hi Footwear etc. Team,
-Quick note regarding Footwear etc.—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
+          <t>Hi mybest Team,
+Quick note regarding mybest—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -2241,13 +2261,13 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Footwear etc. (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for mybest (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Hi Footwear etc. Team,
-I put together a quick technical audit for Footwear etc.. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
+          <t>Hi mybest Team,
+I put together a quick technical audit for mybest. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -2256,13 +2276,13 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>2-min video for Footwear etc.?</t>
+          <t>2-min video for mybest?</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>Hi Footwear etc. Team,
-Spotted a quick fix on Footwear etc.'s checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
+          <t>Hi mybest Team,
+Spotted a quick fix on mybest's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -2270,12 +2290,12 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Footwear etc.. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Footwear etc.—would love to connect!</t>
+          <t>Hi there, love what you're building at mybest. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for mybest—would love to connect!</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Footwear etc.. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at mybest. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -2292,12 +2312,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>StartUs Insights</t>
+          <t>BEST Express Vietnam</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://startus-insights.com</t>
+          <t>https://sale.best-inc.vn</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2305,31 +2325,43 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>zlibjs@0.3.1</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Undeliverable Domain</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>19001031</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>@bestexpressvietnam</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/bestexpressvietnam/</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/bestexpressvietnam/</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>WooCommerce / WordPress</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>1546</v>
+        <v>1724</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
@@ -2354,33 +2386,33 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1546ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1724ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>Idea for StartUs Insights (scaled US store to 4.89% CVR)</t>
+          <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>Hi StartUs Insights Team,
-Love what you've built with StartUs Insights—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+          <t>Hi BEST Express Vietnam Team,
+Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for StartUs Insights?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express Vietnam?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>Quick observation on StartUs Insights's conversion &amp; tracking</t>
+          <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Hi StartUs Insights Team,
-Quick note regarding StartUs Insights—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi BEST Express Vietnam Team,
+Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -2389,13 +2421,13 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>Quick CRO fix for StartUs Insights (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Hi StartUs Insights Team,
-I put together a quick technical audit for StartUs Insights. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi BEST Express Vietnam Team,
+I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -2404,13 +2436,13 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>2-min video for StartUs Insights?</t>
+          <t>2-min video for BEST Express Vietnam?</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>Hi StartUs Insights Team,
-Spotted a quick fix on StartUs Insights's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi BEST Express Vietnam Team,
+Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -2418,12 +2450,12 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at StartUs Insights. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for StartUs Insights—would love to connect!</t>
+          <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at StartUs Insights. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -2440,12 +2472,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Brand House Direct</t>
+          <t>BEST Express Vietnam</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://brandhousedirect.com.au</t>
+          <t>https://service.best-inc.vn</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2455,7 +2487,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>support@brandhousedirect.com.au</t>
+          <t>mkt-vn-sns@best-inc.com</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2465,7 +2497,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1300735786</t>
+          <t>19001031</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -2473,27 +2505,27 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>@brandhousedirectau</t>
+          <t>@bestexpressvietnam</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/brandhousedirectau/</t>
+          <t>https://www.instagram.com/bestexpressvietnam/</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/brandhousedirect</t>
+          <t>https://www.facebook.com/bestexpressvietnam</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Custom / Headless</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O14" t="n">
-        <v>2323</v>
+        <v>1829</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
@@ -2507,7 +2539,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -2518,33 +2550,33 @@
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2323ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1829ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Idea for Brand House Direct (scaled US store to 4.89% CVR)</t>
+          <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Hi Brand House Direct Team,
-Love what you've built with Brand House Direct—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+          <t>Hi BEST Express Vietnam Team,
+Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Brand House Direct?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express Vietnam?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Quick observation on Brand House Direct's conversion &amp; tracking</t>
+          <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Hi Brand House Direct Team,
-Quick note regarding Brand House Direct—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi BEST Express Vietnam Team,
+Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -2553,13 +2585,13 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Brand House Direct (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Hi Brand House Direct Team,
-I put together a quick technical audit for Brand House Direct. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi BEST Express Vietnam Team,
+I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -2568,13 +2600,13 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>2-min video for Brand House Direct?</t>
+          <t>2-min video for BEST Express Vietnam?</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>Hi Brand House Direct Team,
-Spotted a quick fix on Brand House Direct's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi BEST Express Vietnam Team,
+Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -2582,17 +2614,17 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Brand House Direct. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brand House Direct—would love to connect!</t>
+          <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Brand House Direct. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>New Lead</t>
+          <t>Contacted</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
@@ -2604,12 +2636,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bestbuy</t>
+          <t>BEST Express</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://bestbuy.com</t>
+          <t>https://best-inc.vn</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2617,10 +2649,14 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>fullpage.js@2.9.7</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>No Email</t>
+          <t>Undeliverable Domain</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -2633,15 +2669,15 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Custom / Headless</t>
         </is>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>4226</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2651,7 +2687,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2662,33 +2698,33 @@
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.bestbuy.com', port=4</t>
+          <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4226ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Idea for Bestbuy (scaled US store to 4.89% CVR)</t>
+          <t>Idea for BEST Express (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>Hi Bestbuy Team,
-Love what you've built with Bestbuy—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, leaving easy revenue on the table.
+          <t>Hi BEST Express Team,
+Love what you've built with BEST Express—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
 I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Bestbuy?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for BEST Express?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Quick observation on Bestbuy's conversion &amp; tracking</t>
+          <t>Quick observation on BEST Express's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Hi Bestbuy Team,
-Quick note regarding Bestbuy—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, which might be causing paid traffic to bounce without converting.
+          <t>Hi BEST Express Team,
+Quick note regarding BEST Express—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -2697,13 +2733,13 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Bestbuy (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for BEST Express (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Hi Bestbuy Team,
-I put together a quick technical audit for Bestbuy. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4.
+          <t>Hi BEST Express Team,
+I put together a quick technical audit for BEST Express. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -2712,13 +2748,13 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>2-min video for Bestbuy?</t>
+          <t>2-min video for BEST Express?</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Hi Bestbuy Team,
-Spotted a quick fix on Bestbuy's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4). 
+          <t>Hi BEST Express Team,
+Spotted a quick fix on BEST Express's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -2726,12 +2762,12 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Bestbuy. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Bestbuy—would love to connect!</t>
+          <t>Hi there, love what you're building at BEST Express. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express—would love to connect!</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Bestbuy. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at BEST Express. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -2748,12 +2784,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Myntra</t>
+          <t>Synonyms and Antonyms of Words</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://myntra.com</t>
+          <t>https://thesaurus.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2771,17 +2807,29 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>@dictionarycom</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/dictionarycom</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dictionarycom</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>WooCommerce / WordPress</t>
         </is>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>4121</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
@@ -2795,7 +2843,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>MISSING ❌</t>
+          <t>ACTIVE ✅</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2806,33 +2854,33 @@
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.myntra.com', port=44</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4121ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Idea for Myntra (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Synonyms and Antonyms of Words (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Hi Myntra Team,
-Love what you've built with Myntra—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, leaving easy revenue on the table.
+          <t>Hi Synonyms and Antonyms of Words Team,
+Love what you've built with Synonyms and Antonyms of Words—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Myntra?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Synonyms and Antonyms of Words?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Quick observation on Myntra's conversion &amp; tracking</t>
+          <t>Quick observation on Synonyms and Antonyms of Words's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Hi Myntra Team,
-Quick note regarding Myntra—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, which might be causing paid traffic to bounce without converting.
+          <t>Hi Synonyms and Antonyms of Words Team,
+Quick note regarding Synonyms and Antonyms of Words—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -2841,13 +2889,13 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Myntra (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Synonyms and Antonyms of Words (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Hi Myntra Team,
-I put together a quick technical audit for Myntra. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44.
+          <t>Hi Synonyms and Antonyms of Words Team,
+I put together a quick technical audit for Synonyms and Antonyms of Words. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -2856,13 +2904,13 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>2-min video for Myntra?</t>
+          <t>2-min video for Synonyms and Antonyms of Words?</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Hi Myntra Team,
-Spotted a quick fix on Myntra's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44). 
+          <t>Hi Synonyms and Antonyms of Words Team,
+Spotted a quick fix on Synonyms and Antonyms of Words's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -2870,12 +2918,12 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Myntra. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Myntra—would love to connect!</t>
+          <t>Hi there, love what you're building at Synonyms and Antonyms of Words. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Synonyms and Antonyms of Words—would love to connect!</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Myntra. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Synonyms and Antonyms of Words. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -2892,23 +2940,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Brandname.com</t>
+          <t>Umbrex</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://brandname.com</t>
+          <t>https://umbrex.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Unverified</t>
+          <t>No Email</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -2921,11 +2969,11 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Custom / Headless</t>
         </is>
       </c>
       <c r="O17" t="n">
-        <v>2220</v>
+        <v>4225</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
@@ -2950,15 +2998,759 @@
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr">
         <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4225ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Idea for Umbrex (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+Love what you've built with Umbrex—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Umbrex?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>Quick observation on Umbrex's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+Quick note regarding Umbrex—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Umbrex (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+I put together a quick technical audit for Umbrex. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>2-min video for Umbrex?</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Hi Umbrex Team,
+Spotted a quick fix on Umbrex's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Umbrex. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Umbrex—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Umbrex. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Onlinelibrary</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>970</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Idea for Onlinelibrary (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Love what you've built with Onlinelibrary—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Onlinelibrary?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>Quick observation on Onlinelibrary's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Quick note regarding Onlinelibrary—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Onlinelibrary (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+I put together a quick technical audit for Onlinelibrary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>2-min video for Onlinelibrary?</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Spotted a quick fix on Onlinelibrary's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Onlinelibrary. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Onlinelibrary—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Onlinelibrary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>StartUs Insights</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://startus-insights.com</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>zlibjs@0.3.1</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Undeliverable Domain</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>WooCommerce / WordPress</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>1546</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1546ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Idea for StartUs Insights (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+Love what you've built with StartUs Insights—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for StartUs Insights?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Quick observation on StartUs Insights's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+Quick note regarding StartUs Insights—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for StartUs Insights (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+I put together a quick technical audit for StartUs Insights. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>2-min video for StartUs Insights?</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>Hi StartUs Insights Team,
+Spotted a quick fix on StartUs Insights's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at StartUs Insights. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for StartUs Insights—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at StartUs Insights. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brand House Direct</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://brandhousedirect.com.au</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>support@brandhousedirect.com.au</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1300735786</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>@brandhousedirectau</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/brandhousedirectau/</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/brandhousedirect</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Custom / Headless</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>2323</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2323ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Idea for Brand House Direct (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+Love what you've built with Brand House Direct—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Brand House Direct?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>Quick observation on Brand House Direct's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+Quick note regarding Brand House Direct—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Brand House Direct (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+I put together a quick technical audit for Brand House Direct. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>2-min video for Brand House Direct?</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>Hi Brand House Direct Team,
+Spotted a quick fix on Brand House Direct's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Brand House Direct. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brand House Direct—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Brand House Direct. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Bestbuy</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://bestbuy.com</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.bestbuy.com', port=4</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Idea for Bestbuy (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Love what you've built with Bestbuy—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Bestbuy?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Quick observation on Bestbuy's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Quick note regarding Bestbuy—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Bestbuy (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+I put together a quick technical audit for Bestbuy. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>2-min video for Bestbuy?</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Spotted a quick fix on Bestbuy's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Bestbuy. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Bestbuy—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Bestbuy. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Brandname.com</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://brandname.com</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>2220</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2220ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="V22" t="inlineStr">
         <is>
           <t>Idea for Brandname.com (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 Love what you've built with Brandname.com—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -2968,12 +3760,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>Quick observation on Brandname.com's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 Quick note regarding Brandname.com—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -2983,12 +3775,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="Z22" t="inlineStr">
         <is>
           <t>Quick CRO fix for Brandname.com (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AA22" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 I put together a quick technical audit for Brandname.com. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -2998,12 +3790,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
+      <c r="AB22" t="inlineStr">
         <is>
           <t>2-min video for Brandname.com?</t>
         </is>
       </c>
-      <c r="AC17" t="inlineStr">
+      <c r="AC22" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 Spotted a quick fix on Brandname.com's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -3012,117 +3804,117 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD17" t="inlineStr">
+      <c r="AD22" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Brandname.com. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brandname.com—would love to connect!</t>
         </is>
       </c>
-      <c r="AE17" t="inlineStr">
+      <c r="AE22" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Brandname.com. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF17" t="inlineStr">
+      <c r="AF22" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG17" t="inlineStr">
+      <c r="AG22" t="inlineStr">
         <is>
           <t>2026-08-16 20:54</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>FOOTDISTRICT</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>https://footdistrict.com</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>help@footdistrict.com</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Verified (Deliverable)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
         <is>
           <t>@footdistrict</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>https://www.instagram.com/footdistrict/</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>https://www.facebook.com/footDistrict</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>@footdistrict</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="O18" t="n">
+      <c r="O23" t="n">
         <v>1434</v>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S23" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T23" t="inlineStr">
         <is>
           <t>Trustpilot</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
         <is>
           <t>Idea for FOOTDISTRICT (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 Love what you've built with FOOTDISTRICT—your site design and positioning look great. While auditing the store, I noticed product page social proof and mobile retargeting, leaving easy revenue on the table.
@@ -3132,12 +3924,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>Quick observation on FOOTDISTRICT's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 Quick note regarding FOOTDISTRICT—spotted a quick tracking and conversion gap: product page social proof and mobile retargeting, which might be causing paid traffic to bounce without converting.
@@ -3147,12 +3939,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="Z23" t="inlineStr">
         <is>
           <t>Quick CRO fix for FOOTDISTRICT (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr">
+      <c r="AA23" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 I put together a quick technical audit for FOOTDISTRICT. Your page speed and branding look solid, but you're leaving revenue on the table due to product page social proof and mobile retargeting.
@@ -3162,12 +3954,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
+      <c r="AB23" t="inlineStr">
         <is>
           <t>2-min video for FOOTDISTRICT?</t>
         </is>
       </c>
-      <c r="AC18" t="inlineStr">
+      <c r="AC23" t="inlineStr">
         <is>
           <t>Hi FOOTDISTRICT Team,
 Spotted a quick fix on FOOTDISTRICT's checkout &amp; tracking setup (product page social proof and mobile retargeting). 
@@ -3176,113 +3968,113 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD18" t="inlineStr">
+      <c r="AD23" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at FOOTDISTRICT. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for FOOTDISTRICT—would love to connect!</t>
         </is>
       </c>
-      <c r="AE18" t="inlineStr">
+      <c r="AE23" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at FOOTDISTRICT. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF18" t="inlineStr">
+      <c r="AF23" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="AG18" t="inlineStr">
+      <c r="AG23" t="inlineStr">
         <is>
           <t>2026-08-16 20:51</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>APB</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>https://www.apbstore.com</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>info@apbstore.com</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Verified (Deliverable)</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
         <is>
           <t>@apbstore</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>https://www.instagram.com/apbstore/?hl=en</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>https://www.facebook.com/theapbstore/</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="O19" t="n">
+      <c r="O24" t="n">
         <v>1021</v>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S24" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr">
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
         <is>
           <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>Idea for APB (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>Hi APB Team,
 Love what you've built with APB—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
@@ -3292,12 +4084,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>Quick observation on APB's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>Hi APB Team,
 Quick note regarding APB—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
@@ -3307,12 +4099,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="Z24" t="inlineStr">
         <is>
           <t>Quick CRO fix for APB (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA19" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t>Hi APB Team,
 I put together a quick technical audit for APB. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
@@ -3322,12 +4114,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
+      <c r="AB24" t="inlineStr">
         <is>
           <t>2-min video for APB?</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AC24" t="inlineStr">
         <is>
           <t>Hi APB Team,
 Spotted a quick fix on APB's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
@@ -3336,22 +4128,22 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD19" t="inlineStr">
+      <c r="AD24" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at APB. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for APB—would love to connect!</t>
         </is>
       </c>
-      <c r="AE19" t="inlineStr">
+      <c r="AE24" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at APB. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF19" t="inlineStr">
+      <c r="AF24" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG19" t="inlineStr">
+      <c r="AG24" t="inlineStr">
         <is>
           <t>2026-08-16 20:48</t>
         </is>

</xml_diff>

<commit_message>
Fix Vercel routing: add routes map and auto-resolving apiFetch helper
</commit_message>
<xml_diff>
--- a/output/leads_latest.xlsx
+++ b/output/leads_latest.xlsx
@@ -636,12 +636,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Topcv</t>
+          <t>FOOTDISTRICT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://topcv.vn</t>
+          <t>https://footdistrict.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -649,60 +649,228 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>help@footdistrict.com</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>No Email</t>
+          <t>Verified (Deliverable)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>@footdistrict</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/footdistrict/</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/footDistrict</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>@footdistrict</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>3606</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Trustpilot</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Slow server response time (3606ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Idea for FOOTDISTRICT (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Hi FOOTDISTRICT Team,
+Love what you've built with FOOTDISTRICT—your site design and positioning look great. While auditing the store, I noticed slow server response time (3606ms) hurting mobile conversion rate, leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for FOOTDISTRICT?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Quick observation on FOOTDISTRICT's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Hi FOOTDISTRICT Team,
+Quick note regarding FOOTDISTRICT—spotted a quick tracking and conversion gap: slow server response time (3606ms) hurting mobile conversion rate, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for FOOTDISTRICT (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Hi FOOTDISTRICT Team,
+I put together a quick technical audit for FOOTDISTRICT. Your page speed and branding look solid, but you're leaving revenue on the table due to slow server response time (3606ms) hurting mobile conversion rate.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>2-min video for FOOTDISTRICT?</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Hi FOOTDISTRICT Team,
+Spotted a quick fix on FOOTDISTRICT's checkout &amp; tracking setup (slow server response time (3606ms) hurting mobile conversion rate). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at FOOTDISTRICT. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for FOOTDISTRICT—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at FOOTDISTRICT. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>2026-08-16 21:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Topcv</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://topcv.vn</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Magento</t>
         </is>
       </c>
-      <c r="O2" t="n">
+      <c r="O3" t="n">
         <v>688</v>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
         <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Idea for Topcv (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Hi Topcv Team,
 Love what you've built with Topcv—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -712,12 +880,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>Quick observation on Topcv's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Hi Topcv Team,
 Quick note regarding Topcv—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -727,12 +895,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>Quick CRO fix for Topcv (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Hi Topcv Team,
 I put together a quick technical audit for Topcv. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -742,12 +910,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>2-min video for Topcv?</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>Hi Topcv Team,
 Spotted a quick fix on Topcv's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -756,109 +924,109 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Topcv. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Topcv—would love to connect!</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Topcv. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Cambridge Dictionary</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>https://dictionary.cambridge.org</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>No Email</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>@cambridgewords</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>https://www.instagram.com/cambridgewords</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>https://www.facebook.com/CUPCambridgeDictionary/</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
         <is>
           <t>Magento</t>
         </is>
       </c>
-      <c r="O3" t="n">
+      <c r="O4" t="n">
         <v>917</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr">
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
         <is>
           <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Idea for Cambridge Dictionary (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Hi Cambridge Dictionary Team,
 Love what you've built with Cambridge Dictionary—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
@@ -868,12 +1036,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>Quick observation on Cambridge Dictionary's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Hi Cambridge Dictionary Team,
 Quick note regarding Cambridge Dictionary—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
@@ -883,12 +1051,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>Quick CRO fix for Cambridge Dictionary (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Hi Cambridge Dictionary Team,
 I put together a quick technical audit for Cambridge Dictionary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
@@ -898,12 +1066,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>2-min video for Cambridge Dictionary?</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>Hi Cambridge Dictionary Team,
 Spotted a quick fix on Cambridge Dictionary's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
@@ -912,117 +1080,117 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Cambridge Dictionary. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Cambridge Dictionary—would love to connect!</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Cambridge Dictionary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>2026-08-16 21:19</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Footwear etc.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>https://footwearetc.com</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>privacy@footwearetc.com</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Verified (Deliverable)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>1-800-720-0572</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>@footwearetc</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>https://www.instagram.com/footwearetc/</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>http://www.facebook.com/footwearetc</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
         <is>
           <t>Shopify</t>
         </is>
       </c>
-      <c r="O4" t="n">
+      <c r="O5" t="n">
         <v>3451</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr">
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
         <is>
           <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | Slow server response time (3451ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>Idea for Footwear etc. (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Hi Footwear etc. Team,
 Love what you've built with Footwear etc.—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
@@ -1032,12 +1200,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>Quick observation on Footwear etc.'s conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Hi Footwear etc. Team,
 Quick note regarding Footwear etc.—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
@@ -1047,12 +1215,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>Quick CRO fix for Footwear etc. (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>Hi Footwear etc. Team,
 I put together a quick technical audit for Footwear etc.. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
@@ -1062,12 +1230,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>2-min video for Footwear etc.?</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>Hi Footwear etc. Team,
 Spotted a quick fix on Footwear etc.'s checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
@@ -1076,158 +1244,14 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Footwear etc.. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Footwear etc.—would love to connect!</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Footwear etc.. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>2026-08-16 21:19</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Merriam-webster</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://merriam-webster.com</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>No Email</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Magento</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>3002</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3002ms) hurting mobile conversion rate</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Idea for Merriam-webster (scaled UK brand from £4.6k to £696k+)</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Hi Merriam-webster Team,
-Love what you've built with Merriam-webster—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Merriam-webster?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>Quick observation on Merriam-webster's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>Hi Merriam-webster Team,
-Quick note regarding Merriam-webster—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for Merriam-webster (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>Hi Merriam-webster Team,
-I put together a quick technical audit for Merriam-webster. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>2-min video for Merriam-webster?</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Hi Merriam-webster Team,
-Spotted a quick fix on Merriam-webster's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at Merriam-webster. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Merriam-webster—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at Merriam-webster. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -1244,12 +1268,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Famousfootwear</t>
+          <t>Merriam-webster</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://famousfootwear.com</t>
+          <t>https://merriam-webster.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1277,7 +1301,7 @@
         </is>
       </c>
       <c r="O6" t="n">
-        <v>3322</v>
+        <v>3002</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1302,33 +1326,33 @@
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3322ms) hurting mobile conversion rate</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3002ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Idea for Famousfootwear (scaled UK brand from £4.6k to £696k+)</t>
+          <t>Idea for Merriam-webster (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-Love what you've built with Famousfootwear—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+          <t>Hi Merriam-webster Team,
+Love what you've built with Merriam-webster—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Famousfootwear?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Merriam-webster?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Quick observation on Famousfootwear's conversion &amp; tracking</t>
+          <t>Quick observation on Merriam-webster's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-Quick note regarding Famousfootwear—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Merriam-webster Team,
+Quick note regarding Merriam-webster—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1337,13 +1361,13 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Famousfootwear (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Merriam-webster (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-I put together a quick technical audit for Famousfootwear. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Merriam-webster Team,
+I put together a quick technical audit for Merriam-webster. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1352,13 +1376,13 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2-min video for Famousfootwear?</t>
+          <t>2-min video for Merriam-webster?</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>Hi Famousfootwear Team,
-Spotted a quick fix on Famousfootwear's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Merriam-webster Team,
+Spotted a quick fix on Merriam-webster's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1366,12 +1390,12 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Famousfootwear. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Famousfootwear—would love to connect!</t>
+          <t>Hi there, love what you're building at Merriam-webster. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Merriam-webster—would love to connect!</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Famousfootwear. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Merriam-webster. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1388,12 +1412,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Top Hotel - Official Site</t>
+          <t>Famousfootwear</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://tophotel.com.vn</t>
+          <t>https://famousfootwear.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1401,14 +1425,10 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>tophotel.sales@gmail.com</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Verified (Deliverable)</t>
+          <t>No Email</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -1417,19 +1437,15 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/profile.php?id=100035513540432</t>
-        </is>
-      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>WooCommerce / WordPress</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O7" t="n">
-        <v>4259</v>
+        <v>3322</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -1443,7 +1459,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1454,15 +1470,167 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (3322ms) hurting mobile conversion rate</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Idea for Famousfootwear (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+Love what you've built with Famousfootwear—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Famousfootwear?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Quick observation on Famousfootwear's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+Quick note regarding Famousfootwear—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Famousfootwear (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+I put together a quick technical audit for Famousfootwear. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>2-min video for Famousfootwear?</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Hi Famousfootwear Team,
+Spotted a quick fix on Famousfootwear's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Famousfootwear. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Famousfootwear—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Famousfootwear. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>2026-08-16 21:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Top Hotel - Official Site</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://tophotel.com.vn</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>tophotel.sales@gmail.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Verified (Deliverable)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100035513540432</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>WooCommerce / WordPress</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>4259</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4259ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Idea for Top Hotel - Official Site (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>Hi Top Hotel - Official Site Team,
 Love what you've built with Top Hotel - Official Site—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -1472,12 +1640,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>Quick observation on Top Hotel - Official Site's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>Hi Top Hotel - Official Site Team,
 Quick note regarding Top Hotel - Official Site—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -1487,12 +1655,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>Quick CRO fix for Top Hotel - Official Site (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>Hi Top Hotel - Official Site Team,
 I put together a quick technical audit for Top Hotel - Official Site. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -1502,12 +1670,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AB8" t="inlineStr">
         <is>
           <t>2-min video for Top Hotel - Official Site?</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>Hi Top Hotel - Official Site Team,
 Spotted a quick fix on Top Hotel - Official Site's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -1516,178 +1684,14 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Top Hotel - Official Site. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Top Hotel - Official Site—would love to connect!</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Top Hotel - Official Site. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>2026-08-16 21:19</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Esquire</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://esquire.com</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>editor@esquire.com</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Verified (Deliverable)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>@esquire</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>http://instagram.com/esquire</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/Esquire</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>@esquire</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Magento</t>
-        </is>
-      </c>
-      <c r="O8" t="n">
-        <v>1086</v>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Idea for Esquire (scaled UK brand from £4.6k to £696k+)</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>Hi Esquire Team,
-Love what you've built with Esquire—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Esquire?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>Quick observation on Esquire's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Hi Esquire Team,
-Quick note regarding Esquire—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for Esquire (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>Hi Esquire Team,
-I put together a quick technical audit for Esquire. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>2-min video for Esquire?</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>Hi Esquire Team,
-Spotted a quick fix on Esquire's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at Esquire. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Esquire—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at Esquire. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1704,12 +1708,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ELLE</t>
+          <t>Esquire</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://elle.com</t>
+          <t>https://esquire.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1719,7 +1723,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>contactus@elle.com</t>
+          <t>editor@esquire.com</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1733,22 +1737,22 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>@elleusa</t>
+          <t>@esquire</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>http://instagram.com/elleusa</t>
+          <t>http://instagram.com/esquire</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/ellemagazine</t>
+          <t>https://www.facebook.com/Esquire</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>@ellemagazine</t>
+          <t>@esquire</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1757,7 +1761,7 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>820</v>
+        <v>1086</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
@@ -1787,28 +1791,28 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Idea for ELLE (scaled UK brand from £4.6k to £696k+)</t>
+          <t>Idea for Esquire (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Hi ELLE Team,
-Love what you've built with ELLE—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+          <t>Hi Esquire Team,
+Love what you've built with Esquire—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for ELLE?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Esquire?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Quick observation on ELLE's conversion &amp; tracking</t>
+          <t>Quick observation on Esquire's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Hi ELLE Team,
-Quick note regarding ELLE—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Esquire Team,
+Quick note regarding Esquire—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -1817,13 +1821,13 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>Quick CRO fix for ELLE (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Esquire (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Hi ELLE Team,
-I put together a quick technical audit for ELLE. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Esquire Team,
+I put together a quick technical audit for Esquire. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -1832,13 +1836,13 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2-min video for ELLE?</t>
+          <t>2-min video for Esquire?</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>Hi ELLE Team,
-Spotted a quick fix on ELLE's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Esquire Team,
+Spotted a quick fix on Esquire's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -1846,12 +1850,12 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at ELLE. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for ELLE—would love to connect!</t>
+          <t>Hi there, love what you're building at Esquire. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Esquire—would love to connect!</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at ELLE. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Esquire. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -1868,12 +1872,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tops Market</t>
+          <t>ELLE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://topsmarket.vn</t>
+          <t>https://elle.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1881,10 +1885,14 @@
           <t>UK</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>contactus@elle.com</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>No Email</t>
+          <t>Verified (Deliverable)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1893,27 +1901,31 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>@topsmarketvn</t>
+          <t>@elleusa</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/topsmarketvn/</t>
+          <t>http://instagram.com/elleusa</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/TopsmarketVietnam</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>https://www.facebook.com/ellemagazine</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>@ellemagazine</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>WooCommerce / WordPress</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O10" t="n">
-        <v>1297</v>
+        <v>820</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1927,7 +1939,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1938,15 +1950,171 @@
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Idea for ELLE (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Hi ELLE Team,
+Love what you've built with ELLE—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for ELLE?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Quick observation on ELLE's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Hi ELLE Team,
+Quick note regarding ELLE—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for ELLE (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Hi ELLE Team,
+I put together a quick technical audit for ELLE. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>2-min video for ELLE?</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Hi ELLE Team,
+Spotted a quick fix on ELLE's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at ELLE. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for ELLE—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at ELLE. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>2026-08-16 21:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tops Market</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://topsmarket.vn</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>@topsmarketvn</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/topsmarketvn/</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/TopsmarketVietnam</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>WooCommerce / WordPress</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>1297</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>Idea for Tops Market (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>Hi Tops Market Team,
 Love what you've built with Tops Market—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -1956,12 +2124,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>Quick observation on Tops Market's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Hi Tops Market Team,
 Quick note regarding Tops Market—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -1971,12 +2139,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>Quick CRO fix for Tops Market (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>Hi Tops Market Team,
 I put together a quick technical audit for Tops Market. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -1986,12 +2154,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AB11" t="inlineStr">
         <is>
           <t>2-min video for Tops Market?</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>Hi Tops Market Team,
 Spotted a quick fix on Tops Market's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -2000,158 +2168,14 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD10" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Tops Market. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Tops Market—would love to connect!</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr">
+      <c r="AE11" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Tops Market. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF10" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>2026-08-16 21:19</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Myntra</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://myntra.com</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>No Email</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.myntra.com', port=44</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Idea for Myntra (scaled UK brand from £4.6k to £696k+)</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>Hi Myntra Team,
-Love what you've built with Myntra—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, leaving easy revenue on the table.
-I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Myntra?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>Quick observation on Myntra's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Hi Myntra Team,
-Quick note regarding Myntra—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for Myntra (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>Hi Myntra Team,
-I put together a quick technical audit for Myntra. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44.
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>2-min video for Myntra?</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>Hi Myntra Team,
-Spotted a quick fix on Myntra's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at Myntra. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Myntra—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at Myntra. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -2168,17 +2192,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mybest</t>
+          <t>Myntra</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://vn.my-best.com</t>
+          <t>https://myntra.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -2197,11 +2221,11 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O12" t="n">
-        <v>1533</v>
+        <v>0</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -2215,7 +2239,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -2226,15 +2250,159 @@
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.myntra.com', port=44</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Idea for Myntra (scaled UK brand from £4.6k to £696k+)</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+Love what you've built with Myntra—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, leaving easy revenue on the table.
+I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Myntra?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Quick observation on Myntra's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+Quick note regarding Myntra—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Myntra (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+I put together a quick technical audit for Myntra. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>2-min video for Myntra?</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>Hi Myntra Team,
+Spotted a quick fix on Myntra's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.myntra.com', port=44). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Myntra. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Myntra—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Myntra. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>2026-08-16 21:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mybest</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://vn.my-best.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No Email</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>1533</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1533ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>Idea for mybest (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>Hi mybest Team,
 Love what you've built with mybest—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -2244,12 +2412,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>Quick observation on mybest's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>Hi mybest Team,
 Quick note regarding mybest—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -2259,12 +2427,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>Quick CRO fix for mybest (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA13" t="inlineStr">
         <is>
           <t>Hi mybest Team,
 I put together a quick technical audit for mybest. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -2274,12 +2442,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB13" t="inlineStr">
         <is>
           <t>2-min video for mybest?</t>
         </is>
       </c>
-      <c r="AC12" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>Hi mybest Team,
 Spotted a quick fix on mybest's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -2288,113 +2456,113 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr">
+      <c r="AD13" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at mybest. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for mybest—would love to connect!</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
+      <c r="AE13" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at mybest. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF12" t="inlineStr">
+      <c r="AF13" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG12" t="inlineStr">
+      <c r="AG13" t="inlineStr">
         <is>
           <t>2026-08-16 20:59</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>BEST Express Vietnam</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>https://sale.best-inc.vn</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
         <is>
           <t>No Email</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>19001031</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>@bestexpressvietnam</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>https://www.instagram.com/bestexpressvietnam/</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>https://www.facebook.com/bestexpressvietnam/</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
         <is>
           <t>Magento</t>
         </is>
       </c>
-      <c r="O13" t="n">
+      <c r="O14" t="n">
         <v>1724</v>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr">
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
         <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1724ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -2404,12 +2572,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -2419,12 +2587,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA13" t="inlineStr">
+      <c r="AA14" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -2434,12 +2602,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
+      <c r="AB14" t="inlineStr">
         <is>
           <t>2-min video for BEST Express Vietnam?</t>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -2448,117 +2616,117 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD13" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
         </is>
       </c>
-      <c r="AE13" t="inlineStr">
+      <c r="AE14" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF13" t="inlineStr">
+      <c r="AF14" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG13" t="inlineStr">
+      <c r="AG14" t="inlineStr">
         <is>
           <t>2026-08-16 20:59</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>BEST Express Vietnam</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>https://service.best-inc.vn</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>mkt-vn-sns@best-inc.com</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Verified (Deliverable)</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>19001031</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
         <is>
           <t>@bestexpressvietnam</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>https://www.instagram.com/bestexpressvietnam/</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>https://www.facebook.com/bestexpressvietnam</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
         <is>
           <t>Magento</t>
         </is>
       </c>
-      <c r="O14" t="n">
+      <c r="O15" t="n">
         <v>1829</v>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
         <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1829ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>Idea for BEST Express Vietnam (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 Love what you've built with BEST Express Vietnam—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -2568,12 +2736,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>Quick observation on BEST Express Vietnam's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 Quick note regarding BEST Express Vietnam—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -2583,12 +2751,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>Quick CRO fix for BEST Express Vietnam (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA14" t="inlineStr">
+      <c r="AA15" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 I put together a quick technical audit for BEST Express Vietnam. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -2598,12 +2766,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
+      <c r="AB15" t="inlineStr">
         <is>
           <t>2-min video for BEST Express Vietnam?</t>
         </is>
       </c>
-      <c r="AC14" t="inlineStr">
+      <c r="AC15" t="inlineStr">
         <is>
           <t>Hi BEST Express Vietnam Team,
 Spotted a quick fix on BEST Express Vietnam's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -2612,101 +2780,101 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD14" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at BEST Express Vietnam. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express Vietnam—would love to connect!</t>
         </is>
       </c>
-      <c r="AE14" t="inlineStr">
+      <c r="AE15" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at BEST Express Vietnam. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF14" t="inlineStr">
+      <c r="AF15" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="AG14" t="inlineStr">
+      <c r="AG15" t="inlineStr">
         <is>
           <t>2026-08-16 20:59</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>BEST Express</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>https://best-inc.vn</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>fullpage.js@2.9.7</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Undeliverable Domain</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
         <is>
           <t>Custom / Headless</t>
         </is>
       </c>
-      <c r="O15" t="n">
+      <c r="O16" t="n">
         <v>4226</v>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr">
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
         <is>
           <t>Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4226ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>Idea for BEST Express (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>Hi BEST Express Team,
 Love what you've built with BEST Express—your site design and positioning look great. While auditing the store, I noticed missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), leaving easy revenue on the table.
@@ -2716,12 +2884,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>Quick observation on BEST Express's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>Hi BEST Express Team,
 Quick note regarding BEST Express—spotted a quick tracking and conversion gap: missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads), which might be causing paid traffic to bounce without converting.
@@ -2731,12 +2899,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>Quick CRO fix for BEST Express (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>Hi BEST Express Team,
 I put together a quick technical audit for BEST Express. Your page speed and branding look solid, but you're leaving revenue on the table due to missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads).
@@ -2746,12 +2914,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
+      <c r="AB16" t="inlineStr">
         <is>
           <t>2-min video for BEST Express?</t>
         </is>
       </c>
-      <c r="AC15" t="inlineStr">
+      <c r="AC16" t="inlineStr">
         <is>
           <t>Hi BEST Express Team,
 Spotted a quick fix on BEST Express's checkout &amp; tracking setup (missing tiktok pixel (losing out on tiktok ad retargeting &amp; catalog ads)). 
@@ -2760,109 +2928,109 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD15" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at BEST Express. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for BEST Express—would love to connect!</t>
         </is>
       </c>
-      <c r="AE15" t="inlineStr">
+      <c r="AE16" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at BEST Express. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF15" t="inlineStr">
+      <c r="AF16" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG15" t="inlineStr">
+      <c r="AG16" t="inlineStr">
         <is>
           <t>2026-08-16 20:59</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Synonyms and Antonyms of Words</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>https://thesaurus.com</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
         <is>
           <t>No Email</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
         <is>
           <t>@dictionarycom</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>https://www.instagram.com/dictionarycom</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>https://www.facebook.com/dictionarycom</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
         <is>
           <t>WooCommerce / WordPress</t>
         </is>
       </c>
-      <c r="O16" t="n">
+      <c r="O17" t="n">
         <v>4121</v>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
         <is>
           <t>ACTIVE ✅</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
         <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4121ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>Idea for Synonyms and Antonyms of Words (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>Hi Synonyms and Antonyms of Words Team,
 Love what you've built with Synonyms and Antonyms of Words—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -2872,12 +3040,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>Quick observation on Synonyms and Antonyms of Words's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>Hi Synonyms and Antonyms of Words Team,
 Quick note regarding Synonyms and Antonyms of Words—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -2887,12 +3055,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr">
+      <c r="Z17" t="inlineStr">
         <is>
           <t>Quick CRO fix for Synonyms and Antonyms of Words (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA16" t="inlineStr">
+      <c r="AA17" t="inlineStr">
         <is>
           <t>Hi Synonyms and Antonyms of Words Team,
 I put together a quick technical audit for Synonyms and Antonyms of Words. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -2902,12 +3070,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
+      <c r="AB17" t="inlineStr">
         <is>
           <t>2-min video for Synonyms and Antonyms of Words?</t>
         </is>
       </c>
-      <c r="AC16" t="inlineStr">
+      <c r="AC17" t="inlineStr">
         <is>
           <t>Hi Synonyms and Antonyms of Words Team,
 Spotted a quick fix on Synonyms and Antonyms of Words's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -2916,158 +3084,14 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD16" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Synonyms and Antonyms of Words. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Synonyms and Antonyms of Words—would love to connect!</t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr">
+      <c r="AE17" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Synonyms and Antonyms of Words. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF16" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>2026-08-16 20:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Umbrex</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>https://umbrex.com</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>No Email</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Custom / Headless</t>
-        </is>
-      </c>
-      <c r="O17" t="n">
-        <v>4225</v>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4225ms) hurting mobile conversion rate</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>Idea for Umbrex (scaled US store to 4.89% CVR)</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>Hi Umbrex Team,
-Love what you've built with Umbrex—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Umbrex?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>Quick observation on Umbrex's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>Hi Umbrex Team,
-Quick note regarding Umbrex—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z17" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for Umbrex (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA17" t="inlineStr">
-        <is>
-          <t>Hi Umbrex Team,
-I put together a quick technical audit for Umbrex. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB17" t="inlineStr">
-        <is>
-          <t>2-min video for Umbrex?</t>
-        </is>
-      </c>
-      <c r="AC17" t="inlineStr">
-        <is>
-          <t>Hi Umbrex Team,
-Spotted a quick fix on Umbrex's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD17" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at Umbrex. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Umbrex—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at Umbrex. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -3084,12 +3108,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Onlinelibrary</t>
+          <t>Umbrex</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com</t>
+          <t>https://umbrex.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3113,11 +3137,11 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Custom / Headless</t>
         </is>
       </c>
       <c r="O18" t="n">
-        <v>970</v>
+        <v>4225</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -3142,33 +3166,33 @@
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (4225ms) hurting mobile conversion rate</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Idea for Onlinelibrary (scaled US store to 4.89% CVR)</t>
+          <t>Idea for Umbrex (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-Love what you've built with Onlinelibrary—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+          <t>Hi Umbrex Team,
+Love what you've built with Umbrex—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
 I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Onlinelibrary?
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Umbrex?
 Best,
 Talha</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Quick observation on Onlinelibrary's conversion &amp; tracking</t>
+          <t>Quick observation on Umbrex's conversion &amp; tracking</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-Quick note regarding Onlinelibrary—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+          <t>Hi Umbrex Team,
+Quick note regarding Umbrex—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
 Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
 Open to a 2-minute video breakdown of how to plug this leak?
 Best,
@@ -3177,13 +3201,13 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>Quick CRO fix for Onlinelibrary (hit £88k/mo with this)</t>
+          <t>Quick CRO fix for Umbrex (hit £88k/mo with this)</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-I put together a quick technical audit for Onlinelibrary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+          <t>Hi Umbrex Team,
+I put together a quick technical audit for Umbrex. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
 Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
 Would you be open to seeing a 2-minute video walkthrough?
 Best,
@@ -3192,13 +3216,13 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>2-min video for Onlinelibrary?</t>
+          <t>2-min video for Umbrex?</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>Hi Onlinelibrary Team,
-Spotted a quick fix on Onlinelibrary's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+          <t>Hi Umbrex Team,
+Spotted a quick fix on Umbrex's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
 Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
 Best,
 Talha</t>
@@ -3206,12 +3230,12 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>Hi there, love what you're building at Onlinelibrary. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Onlinelibrary—would love to connect!</t>
+          <t>Hi there, love what you're building at Umbrex. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Umbrex—would love to connect!</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>Hey team! Love the vibe at Onlinelibrary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+          <t>Hey team! Love the vibe at Umbrex. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -3228,12 +3252,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>StartUs Insights</t>
+          <t>Onlinelibrary</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://startus-insights.com</t>
+          <t>https://onlinelibrary.wiley.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3241,14 +3265,10 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>zlibjs@0.3.1</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Undeliverable Domain</t>
+          <t>No Email</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -3261,11 +3281,11 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>WooCommerce / WordPress</t>
+          <t>Magento</t>
         </is>
       </c>
       <c r="O19" t="n">
-        <v>1546</v>
+        <v>970</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -3279,7 +3299,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>ACTIVE ✅</t>
+          <t>MISSING ❌</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -3290,15 +3310,163 @@
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr">
         <is>
+          <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue)</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Idea for Onlinelibrary (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Love what you've built with Onlinelibrary—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Onlinelibrary?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Quick observation on Onlinelibrary's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Quick note regarding Onlinelibrary—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Onlinelibrary (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+I put together a quick technical audit for Onlinelibrary. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>2-min video for Onlinelibrary?</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>Hi Onlinelibrary Team,
+Spotted a quick fix on Onlinelibrary's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Onlinelibrary. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Onlinelibrary—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Onlinelibrary. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>StartUs Insights</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://startus-insights.com</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>zlibjs@0.3.1</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Undeliverable Domain</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>WooCommerce / WordPress</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>1546</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>ACTIVE ✅</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (1546ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>Idea for StartUs Insights (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>Hi StartUs Insights Team,
 Love what you've built with StartUs Insights—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -3308,12 +3476,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>Quick observation on StartUs Insights's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>Hi StartUs Insights Team,
 Quick note regarding StartUs Insights—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -3323,12 +3491,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="Z20" t="inlineStr">
         <is>
           <t>Quick CRO fix for StartUs Insights (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA19" t="inlineStr">
+      <c r="AA20" t="inlineStr">
         <is>
           <t>Hi StartUs Insights Team,
 I put together a quick technical audit for StartUs Insights. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -3338,12 +3506,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
+      <c r="AB20" t="inlineStr">
         <is>
           <t>2-min video for StartUs Insights?</t>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
+      <c r="AC20" t="inlineStr">
         <is>
           <t>Hi StartUs Insights Team,
 Spotted a quick fix on StartUs Insights's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -3352,117 +3520,117 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD19" t="inlineStr">
+      <c r="AD20" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at StartUs Insights. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for StartUs Insights—would love to connect!</t>
         </is>
       </c>
-      <c r="AE19" t="inlineStr">
+      <c r="AE20" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at StartUs Insights. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF19" t="inlineStr">
+      <c r="AF20" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG19" t="inlineStr">
+      <c r="AG20" t="inlineStr">
         <is>
           <t>2026-08-16 20:59</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Brand House Direct</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>https://brandhousedirect.com.au</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>support@brandhousedirect.com.au</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Verified (Deliverable)</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>1300735786</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
         <is>
           <t>@brandhousedirectau</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>https://www.instagram.com/brandhousedirectau/</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>https://www.facebook.com/brandhousedirect</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
         <is>
           <t>Custom / Headless</t>
         </is>
       </c>
-      <c r="O20" t="n">
+      <c r="O21" t="n">
         <v>2323</v>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr">
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
         <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2323ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>Idea for Brand House Direct (scaled US store to 4.89% CVR)</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>Hi Brand House Direct Team,
 Love what you've built with Brand House Direct—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -3472,12 +3640,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>Quick observation on Brand House Direct's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>Hi Brand House Direct Team,
 Quick note regarding Brand House Direct—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -3487,12 +3655,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="Z21" t="inlineStr">
         <is>
           <t>Quick CRO fix for Brand House Direct (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t>Hi Brand House Direct Team,
 I put together a quick technical audit for Brand House Direct. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -3502,12 +3670,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB20" t="inlineStr">
+      <c r="AB21" t="inlineStr">
         <is>
           <t>2-min video for Brand House Direct?</t>
         </is>
       </c>
-      <c r="AC20" t="inlineStr">
+      <c r="AC21" t="inlineStr">
         <is>
           <t>Hi Brand House Direct Team,
 Spotted a quick fix on Brand House Direct's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -3516,158 +3684,14 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD20" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Brand House Direct. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brand House Direct—would love to connect!</t>
         </is>
       </c>
-      <c r="AE20" t="inlineStr">
+      <c r="AE21" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Brand House Direct. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF20" t="inlineStr">
-        <is>
-          <t>New Lead</t>
-        </is>
-      </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>2026-08-16 20:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Bestbuy</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://bestbuy.com</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>No Email</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>MISSING ❌</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.bestbuy.com', port=4</t>
-        </is>
-      </c>
-      <c r="V21" t="inlineStr">
-        <is>
-          <t>Idea for Bestbuy (scaled US store to 4.89% CVR)</t>
-        </is>
-      </c>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>Hi Bestbuy Team,
-Love what you've built with Bestbuy—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, leaving easy revenue on the table.
-I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Bestbuy?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>Quick observation on Bestbuy's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>Hi Bestbuy Team,
-Quick note regarding Bestbuy—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z21" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for Bestbuy (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>Hi Bestbuy Team,
-I put together a quick technical audit for Bestbuy. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4.
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB21" t="inlineStr">
-        <is>
-          <t>2-min video for Bestbuy?</t>
-        </is>
-      </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>Hi Bestbuy Team,
-Spotted a quick fix on Bestbuy's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at Bestbuy. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Bestbuy—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE21" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at Bestbuy. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -3684,23 +3708,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Brandname.com</t>
+          <t>Bestbuy</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://brandname.com</t>
+          <t>https://bestbuy.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Unverified</t>
+          <t>No Email</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -3713,11 +3737,11 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Magento</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O22" t="n">
-        <v>2220</v>
+        <v>0</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
@@ -3742,15 +3766,159 @@
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr">
         <is>
+          <t>Could not connect or site timed out: HTTPSConnectionPool(host='www.bestbuy.com', port=4</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Idea for Bestbuy (scaled US store to 4.89% CVR)</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Love what you've built with Bestbuy—your site design and positioning look great. While auditing the store, I noticed could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, leaving easy revenue on the table.
+I recently scaled a US D2C store to $34k+ across 569 orders at a 4.89% conversion rate ($59 AOV) by plugging tracking leaks and dialing in paid search.
+Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for Bestbuy?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Quick observation on Bestbuy's conversion &amp; tracking</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Quick note regarding Bestbuy—spotted a quick tracking and conversion gap: could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4, which might be causing paid traffic to bounce without converting.
+Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
+Open to a 2-minute video breakdown of how to plug this leak?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Quick CRO fix for Bestbuy (hit £88k/mo with this)</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+I put together a quick technical audit for Bestbuy. Your page speed and branding look solid, but you're leaving revenue on the table due to could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4.
+Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
+Would you be open to seeing a 2-minute video walkthrough?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>2-min video for Bestbuy?</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>Hi Bestbuy Team,
+Spotted a quick fix on Bestbuy's checkout &amp; tracking setup (could not connect or site timed out: httpsconnectionpool(host='www.bestbuy.com', port=4). 
+Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
+Best,
+Talha</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Hi there, love what you're building at Bestbuy. Recently scaled US store to 4.89% CVR by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Bestbuy—would love to connect!</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>Hey team! Love the vibe at Bestbuy. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>New Lead</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>2026-08-16 20:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Brandname.com</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://brandname.com</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Magento</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>2220</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>MISSING ❌</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
           <t>Missing Meta Pixel / CAPI tracking (blind ad spend on FB &amp; IG) | Missing TikTok Pixel (losing out on TikTok ad retargeting &amp; catalog ads) | No Google Analytics 4 / GTM detected | No structured review / social proof app detected on product pages | No automated email retention (Klaviyo) detected (losing cart recovery revenue) | Slow server response time (2220ms) hurting mobile conversion rate</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>Idea for Brandname.com (scaled UK brand from £4.6k to £696k+)</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 Love what you've built with Brandname.com—your site design and positioning look great. While auditing the store, I noticed missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), leaving easy revenue on the table.
@@ -3760,12 +3928,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>Quick observation on Brandname.com's conversion &amp; tracking</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 Quick note regarding Brandname.com—spotted a quick tracking and conversion gap: missing meta pixel / capi tracking (blind ad spend on fb &amp; ig), which might be causing paid traffic to bounce without converting.
@@ -3775,12 +3943,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="Z23" t="inlineStr">
         <is>
           <t>Quick CRO fix for Brandname.com (hit £88k/mo with this)</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AA23" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 I put together a quick technical audit for Brandname.com. Your page speed and branding look solid, but you're leaving revenue on the table due to missing meta pixel / capi tracking (blind ad spend on fb &amp; ig).
@@ -3790,12 +3958,12 @@
 Talha</t>
         </is>
       </c>
-      <c r="AB22" t="inlineStr">
+      <c r="AB23" t="inlineStr">
         <is>
           <t>2-min video for Brandname.com?</t>
         </is>
       </c>
-      <c r="AC22" t="inlineStr">
+      <c r="AC23" t="inlineStr">
         <is>
           <t>Hi Brandname.com Team,
 Spotted a quick fix on Brandname.com's checkout &amp; tracking setup (missing meta pixel / capi tracking (blind ad spend on fb &amp; ig)). 
@@ -3804,188 +3972,24 @@
 Talha</t>
         </is>
       </c>
-      <c r="AD22" t="inlineStr">
+      <c r="AD23" t="inlineStr">
         <is>
           <t>Hi there, love what you're building at Brandname.com. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for Brandname.com—would love to connect!</t>
         </is>
       </c>
-      <c r="AE22" t="inlineStr">
+      <c r="AE23" t="inlineStr">
         <is>
           <t>Hey team! Love the vibe at Brandname.com. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
         </is>
       </c>
-      <c r="AF22" t="inlineStr">
+      <c r="AF23" t="inlineStr">
         <is>
           <t>New Lead</t>
         </is>
       </c>
-      <c r="AG22" t="inlineStr">
+      <c r="AG23" t="inlineStr">
         <is>
           <t>2026-08-16 20:54</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>FOOTDISTRICT</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>https://footdistrict.com</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>help@footdistrict.com</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Verified (Deliverable)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>@footdistrict</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/footdistrict/</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/footDistrict</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>@footdistrict</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Shopify</t>
-        </is>
-      </c>
-      <c r="O23" t="n">
-        <v>1434</v>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>ACTIVE ✅</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>ACTIVE ✅</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>ACTIVE ✅</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>ACTIVE ✅</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Trustpilot</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
-        <is>
-          <t>Idea for FOOTDISTRICT (scaled UK brand from £4.6k to £696k+)</t>
-        </is>
-      </c>
-      <c r="W23" t="inlineStr">
-        <is>
-          <t>Hi FOOTDISTRICT Team,
-Love what you've built with FOOTDISTRICT—your site design and positioning look great. While auditing the store, I noticed product page social proof and mobile retargeting, leaving easy revenue on the table.
-I recently scaled a UK athletic &amp; lifestyle brand from £4.6k to £696,643.80 (+14,752% growth, £88k in a single month) at a 4.89% CVR and 3.8x ROAS.
-Mind if I send over a quick 2-minute video breakdown showing 2 simple tweaks you can make to fix this for FOOTDISTRICT?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>Quick observation on FOOTDISTRICT's conversion &amp; tracking</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>Hi FOOTDISTRICT Team,
-Quick note regarding FOOTDISTRICT—spotted a quick tracking and conversion gap: product page social proof and mobile retargeting, which might be causing paid traffic to bounce without converting.
-Fixing these exact tracking and checkout leaks helped our UK e-commerce partner reach £206k+ YTD (+65% YoY) with a 3.8x ROAS.
-Open to a 2-minute video breakdown of how to plug this leak?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>Quick CRO fix for FOOTDISTRICT (hit £88k/mo with this)</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>Hi FOOTDISTRICT Team,
-I put together a quick technical audit for FOOTDISTRICT. Your page speed and branding look solid, but you're leaving revenue on the table due to product page social proof and mobile retargeting.
-Dialing in this exact checkout and ad optimization helped us hit £88,048 in a single month at a 4.89% conversion rate.
-Would you be open to seeing a 2-minute video walkthrough?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AB23" t="inlineStr">
-        <is>
-          <t>2-min video for FOOTDISTRICT?</t>
-        </is>
-      </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>Hi FOOTDISTRICT Team,
-Spotted a quick fix on FOOTDISTRICT's checkout &amp; tracking setup (product page social proof and mobile retargeting). 
-Recently scaled a similar store to £696k+ by solving this exact issue. Mind if I send a 2-min video showing how to fix it?
-Best,
-Talha</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>Hi there, love what you're building at FOOTDISTRICT. Recently scaled UK brand from £4.6k to £696k+ by dialing in CRO &amp; tracking. Spotted a quick growth opportunity for FOOTDISTRICT—would love to connect!</t>
-        </is>
-      </c>
-      <c r="AE23" t="inlineStr">
-        <is>
-          <t>Hey team! Love the vibe at FOOTDISTRICT. Spotted a quick tracking gap leaking paid traffic. Scaled a similar store to £696k+ recently and made a 2-minute video showing two easy fixes. Mind if I share it here?</t>
-        </is>
-      </c>
-      <c r="AF23" t="inlineStr">
-        <is>
-          <t>Contacted</t>
-        </is>
-      </c>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>2026-08-16 20:51</t>
         </is>
       </c>
     </row>

</xml_diff>